<commit_message>
Plantilla y Portal: columna 'Administración (empresa)' (cambio visual pedido por Zires; el Portal acepta ambos nombres)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plantillas/Plantilla_Oficial_Carga_Morosidad_Lexia.xlsx
+++ b/plantillas/Plantilla_Oficial_Carga_Morosidad_Lexia.xlsx
@@ -740,7 +740,7 @@
     <row r="11">
       <c r="B11" s="32" t="inlineStr">
         <is>
-          <t>El Portal carga los residentes en el condominio que tengas seleccionado arriba al subir el archivo. Las columnas ID_Condominio y Estado_Contacto son informativas.</t>
+          <t>El Portal carga los residentes en el condominio que tengas seleccionado arriba al subir el archivo. Las columnas Administración (empresa) y Estado_Contacto son informativas.</t>
         </is>
       </c>
     </row>
@@ -774,7 +774,7 @@
     <row r="17">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Cuenta bancaria (Banco y CLABE), quién firma los mensajes (Zires Abogados o el nombre de la Administración) y las reglas de enganche y condonación. El ID_Condominio debe coincidir exactamente con el de tu condominio en el Portal. Se sube en el Portal, en "Actualizar datos bancarios y reglas de negociación de tu condominio".</t>
+          <t>Cuenta bancaria (Banco y CLABE), quién firma los mensajes (Zires Abogados o el nombre de la Administración) y las reglas de enganche y condonación. El ID_Condominio es el código de tu condominio en el Portal (te lo da Zires Abogados) y debe coincidir exactamente; en Administración (empresa) va el nombre de tu empresa administradora. Se sube en el Portal, en "Actualizar datos bancarios y reglas de negociación de tu condominio".</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
     <row r="3" ht="30" customHeight="1" s="28">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>ID_Condominio</t>
+          <t>Administración (empresa)</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -1953,7 +1953,7 @@
     <row r="2">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Llena una fila por condominio, solo la primera vez que lo das de alta o cuando cambien sus políticas. Si dejas en blanco Permite_Enganche o Permite_Condonacion, o sus porcentajes, Lexia usa el criterio general por defecto.</t>
+          <t>Llena una fila por condominio, solo la primera vez que lo das de alta o cuando cambien sus políticas. ID_Condominio es el código de tu condominio en el Portal (te lo da Zires Abogados); Administración (empresa) es el nombre de la empresa administradora. Si dejas en blanco Permite_Enganche o Permite_Condonacion, o sus porcentajes, Lexia usa el criterio general por defecto.</t>
         </is>
       </c>
     </row>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="F4" s="18" t="inlineStr">
         <is>
-          <t>Administrador</t>
+          <t>Administración (empresa)</t>
         </is>
       </c>
       <c r="G4" s="18" t="inlineStr">

</xml_diff>